<commit_message>
fix: make bill_month required for payment upload and format as MMM YY
Backend:
- Add missing Carbon import in PaymentService
- Make bill_month column required in payment upload validation
- Reject rows with invalid or missing bill_month instead of picking any bill

Frontend:
- Add formatBillMonth utility for consistent MMM YY display
- Replace formatDate(bill_month) with formatBillMonth in all pages
- Update payment upload instructions to mention bill_month as required
- Regenerate sample Excel with bill_month column
</commit_message>
<xml_diff>
--- a/backend/public/samples/payment_upload_sample.xlsx
+++ b/backend/public/samples/payment_upload_sample.xlsx
@@ -15,11 +15,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
   <si>
     <t>reference_no</t>
   </si>
   <si>
+    <t>bill_month</t>
+  </si>
+  <si>
     <t>voucher_no</t>
   </si>
   <si>
@@ -38,16 +41,22 @@
     <t>payable</t>
   </si>
   <si>
+    <t>amount_paid</t>
+  </si>
+  <si>
     <t>06141261208900</t>
   </si>
   <si>
+    <t>Sep 25</t>
+  </si>
+  <si>
     <t>VCH-001</t>
   </si>
   <si>
     <t>INS-2026-001</t>
   </si>
   <si>
-    <t>Batch A - Sep 2026</t>
+    <t>Batch A</t>
   </si>
   <si>
     <t>2026-09-20</t>
@@ -68,13 +77,16 @@
     <t>06141261142900</t>
   </si>
   <si>
+    <t>Aug 25</t>
+  </si>
+  <si>
     <t>VCH-003</t>
   </si>
   <si>
     <t>INS-2026-002</t>
   </si>
   <si>
-    <t>Batch B - Sep 2026</t>
+    <t>Batch B</t>
   </si>
   <si>
     <t>2026-09-21</t>
@@ -417,19 +429,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="9.283" bestFit="true" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,73 +454,97 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2">
+        <v>1600</v>
+      </c>
+      <c r="I2">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="G2">
-        <v>1600</v>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3">
+        <v>88735</v>
+      </c>
+      <c r="I3">
+        <v>88735</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
         <v>15</v>
       </c>
-      <c r="G3">
-        <v>88735</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4">
+      <c r="H4">
+        <v>1500</v>
+      </c>
+      <c r="I4">
         <v>1500</v>
       </c>
     </row>

</xml_diff>